<commit_message>
Add weekly China vs RoW table and chart to soybean inspections workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017P77ZfwM5SjirqZevrNVTE
</commit_message>
<xml_diff>
--- a/Soybean_Inspections_Sep_Oct_2025_vs_2026_China_vs_ROW_upd_W4Oct_by_country.xlsx
+++ b/Soybean_Inspections_Sep_Oct_2025_vs_2026_China_vs_ROW_upd_W4Oct_by_country.xlsx
@@ -10,11 +10,12 @@
   <sheets>
     <sheet name="Summary China vs RoW" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Country by Country" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="September" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Week 1 October" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Week 2 October" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Week 3 October" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Week 4 October" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Weekly China vs RoW" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="September" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Week 1 October" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Week 2 October" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Week 3 October" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Week 4 October" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="125">
   <si>
     <t xml:space="preserve">US Soybean Export Inspections — China vs Rest of World (weekly-report basis)</t>
   </si>
@@ -287,6 +288,93 @@
   </si>
   <si>
     <t xml:space="preserve"># countries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US Soybean Export Inspections — China vs Rest of World by week, 2025 vs 2026 (MT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly MT/inspections computed from raw CY2025/CY2026 FGIS files (Grain = SOYBEANS, by "Thursday" week-ending date). Week-ending dates are paired Thursday-to-Thursday (2025 week ends one day later). Check columns must read 0 (tie-out to period tabs).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Week</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w/e 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w/e 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">China 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RoW 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">China 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RoW 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ RoW MT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ RoW %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ Total MT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">China share 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Period tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 Sep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 Sep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17 Sep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 Sep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tie-out check vs period tabs (should be 0):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ Total 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ Total 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ China 2026</t>
   </si>
   <si>
     <t xml:space="preserve">US Soybean Export Inspections — weeks ending Thu 4/11/18/25 Sep 2025 vs Thu 3/10/17/24 Sep 2026 (weekly-report basis)</t>
@@ -320,13 +408,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0;\-#,##0;\-"/>
     <numFmt numFmtId="166" formatCode="\+0.0%;\-0.0%;0.0%"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="dd\-mmm\-yy"/>
+    <numFmt numFmtId="169" formatCode="0;\-0;0"/>
+    <numFmt numFmtId="170" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -390,6 +481,26 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -407,7 +518,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFE5E4E0"/>
       </patternFill>
     </fill>
   </fills>
@@ -445,7 +556,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -522,6 +633,18 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -574,7 +697,7 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF2CC"/>
@@ -582,7 +705,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -593,18 +716,18 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFE5E4E0"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF2A78D6"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FFEB6834"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
@@ -614,10 +737,673 @@
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF1F4E78"/>
-      <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="FF52514E"/>
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Soybean inspections by week: China vs RoW 2026 vs 2025 (MT)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"RoW 2026"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>RoW 2026</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2a78d6"/>
+            </a:solidFill>
+            <a:ln w="19080">
+              <a:solidFill>
+                <a:srgbClr val="ffffff"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Weekly China vs RoW'!$B$5:$B$12</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>3 Sep</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10 Sep</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>17 Sep</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>24 Sep</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1 Oct</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8 Oct</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>15 Oct</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>22 Oct</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Weekly China vs RoW'!$I$5:$I$12</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0;\-#,##0;\-</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>464732</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>352007</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>322909</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>350056</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>442938</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>463342</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>734461</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>824513</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"China 2026"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>China 2026</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="eb6834"/>
+            </a:solidFill>
+            <a:ln w="19080">
+              <a:solidFill>
+                <a:srgbClr val="ffffff"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Weekly China vs RoW'!$B$5:$B$12</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>3 Sep</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10 Sep</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>17 Sep</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>24 Sep</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1 Oct</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8 Oct</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>15 Oct</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>22 Oct</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Weekly China vs RoW'!$H$5:$H$12</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0;\-#,##0;\-</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>328245</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>446789</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>806776</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>756492</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>649252</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1333625</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1651940</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:overlap val="100"/>
+        <c:axId val="77396766"/>
+        <c:axId val="22059041"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"2025 total (all RoW — China 0)"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2025 total (all RoW — China 0)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="52514e"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="52514e"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="52514e"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Weekly China vs RoW'!$B$5:$B$12</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>3 Sep</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10 Sep</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>17 Sep</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>24 Sep</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1 Oct</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8 Oct</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>15 Oct</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>22 Oct</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Weekly China vs RoW'!$G$5:$G$12</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0;\-#,##0;\-</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>467624</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>822666</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>565630</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>610633</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>783495</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1017196</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1591342</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1161105</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:hiLowLines>
+          <c:spPr>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:hiLowLines>
+        <c:marker val="1"/>
+        <c:axId val="77396766"/>
+        <c:axId val="22059041"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="77396766"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Week ending (2026; 2025 week ends one day later)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="22059041"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="22059041"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="e5e4e0"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Metric tons</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="77396766"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>196560</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>107640</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="0" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="4572000"/>
+        <a:ext cx="9359640" cy="4679640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5466,6 +6252,677 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:O21"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="5" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="I4" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="J4" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="K4" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="L4" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="M4" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="N4" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="O4" s="15" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>45904</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>467624</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <f aca="false">E5+F5</f>
+        <v>467624</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>464732</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <f aca="false">H5+I5</f>
+        <v>464732</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <f aca="false">I5-F5</f>
+        <v>-2892</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <f aca="false">IF(F5=0,"new",I5/F5-1)</f>
+        <v>-0.00618445588763628</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <f aca="false">J5-G5</f>
+        <v>-2892</v>
+      </c>
+      <c r="N5" s="8" t="n">
+        <f aca="false">IF(J5=0,0,H5/J5)</f>
+        <v>0</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>45911</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>822666</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <f aca="false">E6+F6</f>
+        <v>822666</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>328245</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>352007</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <f aca="false">H6+I6</f>
+        <v>680252</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <f aca="false">I6-F6</f>
+        <v>-470659</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <f aca="false">IF(F6=0,"new",I6/F6-1)</f>
+        <v>-0.57211432100026</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <f aca="false">J6-G6</f>
+        <v>-142414</v>
+      </c>
+      <c r="N6" s="8" t="n">
+        <f aca="false">IF(J6=0,0,H6/J6)</f>
+        <v>0.482534413717269</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>45918</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>565630</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <f aca="false">E7+F7</f>
+        <v>565630</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>446789</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>322909</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <f aca="false">H7+I7</f>
+        <v>769698</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <f aca="false">I7-F7</f>
+        <v>-242721</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <f aca="false">IF(F7=0,"new",I7/F7-1)</f>
+        <v>-0.429116206707565</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <f aca="false">J7-G7</f>
+        <v>204068</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <f aca="false">IF(J7=0,0,H7/J7)</f>
+        <v>0.580473120626531</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>45925</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>610633</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <f aca="false">E8+F8</f>
+        <v>610633</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>806776</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>350056</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <f aca="false">H8+I8</f>
+        <v>1156832</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <f aca="false">I8-F8</f>
+        <v>-260577</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <f aca="false">IF(F8=0,"new",I8/F8-1)</f>
+        <v>-0.426732587331507</v>
+      </c>
+      <c r="M8" s="6" t="n">
+        <f aca="false">J8-G8</f>
+        <v>546199</v>
+      </c>
+      <c r="N8" s="8" t="n">
+        <f aca="false">IF(J8=0,0,H8/J8)</f>
+        <v>0.697401178390639</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>45932</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>783495</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <f aca="false">E9+F9</f>
+        <v>783495</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>756492</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>442938</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <f aca="false">H9+I9</f>
+        <v>1199430</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <f aca="false">I9-F9</f>
+        <v>-340557</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <f aca="false">IF(F9=0,"new",I9/F9-1)</f>
+        <v>-0.434663909788831</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <f aca="false">J9-G9</f>
+        <v>415935</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <f aca="false">IF(J9=0,0,H9/J9)</f>
+        <v>0.630709587053851</v>
+      </c>
+      <c r="O9" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>45939</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>1017196</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <f aca="false">E10+F10</f>
+        <v>1017196</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>649252</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>463342</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <f aca="false">H10+I10</f>
+        <v>1112594</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <f aca="false">I10-F10</f>
+        <v>-553854</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <f aca="false">IF(F10=0,"new",I10/F10-1)</f>
+        <v>-0.544490933900645</v>
+      </c>
+      <c r="M10" s="6" t="n">
+        <f aca="false">J10-G10</f>
+        <v>95398</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <f aca="false">IF(J10=0,0,H10/J10)</f>
+        <v>0.583547996843413</v>
+      </c>
+      <c r="O10" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>45946</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>1591342</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <f aca="false">E11+F11</f>
+        <v>1591342</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>1333625</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>734461</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <f aca="false">H11+I11</f>
+        <v>2068086</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <f aca="false">I11-F11</f>
+        <v>-856881</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <f aca="false">IF(F11=0,"new",I11/F11-1)</f>
+        <v>-0.538464390432729</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <f aca="false">J11-G11</f>
+        <v>476744</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <f aca="false">IF(J11=0,0,H11/J11)</f>
+        <v>0.644859546459867</v>
+      </c>
+      <c r="O11" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C12" s="19" t="n">
+        <v>45953</v>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>1161105</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <f aca="false">E12+F12</f>
+        <v>1161105</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>1651940</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>824513</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <f aca="false">H12+I12</f>
+        <v>2476453</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <f aca="false">I12-F12</f>
+        <v>-336592</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <f aca="false">IF(F12=0,"new",I12/F12-1)</f>
+        <v>-0.289889372623492</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <f aca="false">J12-G12</f>
+        <v>1315348</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <f aca="false">IF(J12=0,0,H12/J12)</f>
+        <v>0.667058894313762</v>
+      </c>
+      <c r="O12" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="10" t="n">
+        <f aca="false">SUM(E5:E12)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="10" t="n">
+        <f aca="false">SUM(F5:F12)</f>
+        <v>7019691</v>
+      </c>
+      <c r="G13" s="10" t="n">
+        <f aca="false">SUM(G5:G12)</f>
+        <v>7019691</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <f aca="false">SUM(H5:H12)</f>
+        <v>5973119</v>
+      </c>
+      <c r="I13" s="10" t="n">
+        <f aca="false">SUM(I5:I12)</f>
+        <v>3954958</v>
+      </c>
+      <c r="J13" s="10" t="n">
+        <f aca="false">SUM(J5:J12)</f>
+        <v>9928077</v>
+      </c>
+      <c r="K13" s="10" t="n">
+        <f aca="false">SUM(K5:K12)</f>
+        <v>-3064733</v>
+      </c>
+      <c r="L13" s="11" t="n">
+        <f aca="false">IF(F13=0,"new",I13/F13-1)</f>
+        <v>-0.436590869883019</v>
+      </c>
+      <c r="M13" s="10" t="n">
+        <f aca="false">SUM(M5:M12)</f>
+        <v>2908386</v>
+      </c>
+      <c r="N13" s="12" t="n">
+        <f aca="false">IF(J13=0,0,H13/J13)</f>
+        <v>0.601639068673621</v>
+      </c>
+      <c r="O13" s="9"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A17,$G$5:$G$12)-September!B38</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A17,$J$5:$J$12)-September!C38</f>
+        <v>0</v>
+      </c>
+      <c r="D17" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A17,$H$5:$H$12)-September!C39</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A18,$G$5:$G$12)-'Week 1 October'!B30</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A18,$J$5:$J$12)-'Week 1 October'!C30</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A18,$H$5:$H$12)-'Week 1 October'!C31</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A19,$G$5:$G$12)-'Week 2 October'!B31</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A19,$J$5:$J$12)-'Week 2 October'!C31</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A19,$H$5:$H$12)-'Week 2 October'!C32</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A20,$G$5:$G$12)-'Week 3 October'!B30</f>
+        <v>0</v>
+      </c>
+      <c r="C20" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A20,$J$5:$J$12)-'Week 3 October'!C30</f>
+        <v>0</v>
+      </c>
+      <c r="D20" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A20,$H$5:$H$12)-'Week 3 October'!C31</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A21,$G$5:$G$12)-'Week 4 October'!B31</f>
+        <v>0</v>
+      </c>
+      <c r="C21" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A21,$J$5:$J$12)-'Week 4 October'!C31</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="21" t="n">
+        <f aca="false">SUMIF($O$5:$O$12,A21,$H$5:$H$12)-'Week 4 October'!C32</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="K5:M13">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>AND(ISNUMBER(K5),K5&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>AND(ISNUMBER(K5),K5&lt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:H40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -5475,52 +6932,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="19" t="s">
-        <v>89</v>
-      </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
+      <c r="B4" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19"/>
-      <c r="B5" s="20" t="s">
+      <c r="A5" s="22"/>
+      <c r="B5" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="20" t="s">
-        <v>91</v>
+      <c r="H5" s="23" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6582,7 +8039,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -6596,52 +8053,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="19" t="s">
-        <v>89</v>
-      </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
+      <c r="B4" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19"/>
-      <c r="B5" s="20" t="s">
+      <c r="A5" s="22"/>
+      <c r="B5" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="20" t="s">
-        <v>91</v>
+      <c r="H5" s="23" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7471,7 +8928,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -7485,52 +8942,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>93</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="19" t="s">
-        <v>89</v>
-      </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
+      <c r="B4" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19"/>
-      <c r="B5" s="20" t="s">
+      <c r="A5" s="22"/>
+      <c r="B5" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="20" t="s">
-        <v>91</v>
+      <c r="H5" s="23" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8389,7 +9846,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -8403,52 +9860,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="19" t="s">
-        <v>89</v>
-      </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
+      <c r="B4" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19"/>
-      <c r="B5" s="20" t="s">
+      <c r="A5" s="22"/>
+      <c r="B5" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="20" t="s">
-        <v>91</v>
+      <c r="H5" s="23" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9278,7 +10735,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -9292,52 +10749,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>95</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="19" t="s">
-        <v>89</v>
-      </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
+      <c r="B4" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19"/>
-      <c r="B5" s="20" t="s">
+      <c r="A5" s="22"/>
+      <c r="B5" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="20" t="s">
-        <v>91</v>
+      <c r="H5" s="23" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>